<commit_message>
Align Eva_Medoc_Master.xlsx with v4 docx
</commit_message>
<xml_diff>
--- a/data/Eva_Medoc_Master.xlsx
+++ b/data/Eva_Medoc_Master.xlsx
@@ -479,12 +479,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -505,22 +505,22 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Langt løb (km, gang inkl.)</t>
+          <t>Tirsdag</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Run/Walk ratio</t>
+          <t>Torsdag</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Tempo (Tir)</t>
+          <t>Lørdag (lang tur, km)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Status/Note</t>
+          <t>Note</t>
         </is>
       </c>
     </row>
@@ -538,22 +538,24 @@
           <t>Build</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n">
-        <v>8</v>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Løbetur Z2 — 30 min</t>
+        </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>6/2</t>
+          <t>Z2 + strides</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Let Z2</t>
+          <t>8 km</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Z2 base, ingen intervaller endnu</t>
+          <t>Ratio 6/2. Første strides denne uge.</t>
         </is>
       </c>
     </row>
@@ -571,22 +573,24 @@
           <t>Build</t>
         </is>
       </c>
-      <c r="D3" s="2" t="n">
-        <v>10</v>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Løbetur Z2 — 35 min</t>
+        </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>6/2</t>
+          <t>Z2 + strides</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Let Z2</t>
+          <t>10 km</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Z2 base</t>
+          <t>Ratio 6/2, lidt længere.</t>
         </is>
       </c>
     </row>
@@ -604,22 +608,24 @@
           <t>Build</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n">
-        <v>12</v>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Løbetur Z2 — 40 min, ratio 8/2</t>
+        </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>6/2</t>
+          <t>Tempo intervals — intro (3×8 min Z3)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Strides</t>
+          <t>12 km</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Strides fra denne uge</t>
+          <t>Ratio op til 8/2. Første Z3-tempo.</t>
         </is>
       </c>
     </row>
@@ -637,22 +643,24 @@
           <t>Recovery</t>
         </is>
       </c>
-      <c r="D5" s="3" t="n">
-        <v>8</v>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Let løbetur — 25 min</t>
+        </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>6/2</t>
+          <t>Let løbetur — 25 min</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Strides</t>
+          <t>8 km</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Restitution</t>
+          <t>Restitution. Ratio 6/2 eller fri.</t>
         </is>
       </c>
     </row>
@@ -670,22 +678,24 @@
           <t>Build</t>
         </is>
       </c>
-      <c r="D6" s="2" t="n">
-        <v>15</v>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Løbetur Z2 — 40 min, ratio 8/2</t>
+        </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>8/2</t>
+          <t>Tempo intervals (3×10 min Z3)</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Strides</t>
+          <t>14 km</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Ratio op til 8/2</t>
+          <t>Block 2 starter.</t>
         </is>
       </c>
     </row>
@@ -703,20 +713,26 @@
           <t>Build</t>
         </is>
       </c>
-      <c r="D7" s="2" t="n">
-        <v>16</v>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Løbetur Z2 — 45 min, ratio 8/2</t>
+        </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>8/2</t>
+          <t>Tempo intervals progression (4×8 min Z3)</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Strides</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr"/>
+          <t>16 km</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Første gang over 15 km.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -732,22 +748,24 @@
           <t>Build</t>
         </is>
       </c>
-      <c r="D8" s="2" t="n">
-        <v>18</v>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Løbetur Z2 — 45 min, ratio 10/2</t>
+        </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>8/2</t>
+          <t>Tempo intervals progression (3×12 min Z3)</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Tempo-int.</t>
+          <t>18 km</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Tempo-intervaller fra denne uge (tirsdag)</t>
+          <t>Test ratio 10/2 på tirsdag.</t>
         </is>
       </c>
     </row>
@@ -765,22 +783,24 @@
           <t>Recovery</t>
         </is>
       </c>
-      <c r="D9" s="3" t="n">
-        <v>12</v>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Let løbetur — 30 min, ratio 8/2</t>
+        </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>8/2</t>
+          <t>Let løbetur — 30 min</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Tempo-int.</t>
+          <t>12 km</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Restitution</t>
+          <t>Absorber block 2 (14-16-18 km).</t>
         </is>
       </c>
     </row>
@@ -798,22 +818,24 @@
           <t>Build</t>
         </is>
       </c>
-      <c r="D10" s="2" t="n">
-        <v>22</v>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Løbetur Z2 — 50 min, ratio 10/2</t>
+        </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>10/2</t>
+          <t>Marathon pace — intro (20 min)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Tempo-int.</t>
+          <t>20 km</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Ratio op til 10/2</t>
+          <t>Første gang over 18 km.</t>
         </is>
       </c>
     </row>
@@ -831,55 +853,59 @@
           <t>Build</t>
         </is>
       </c>
-      <c r="D11" s="2" t="n">
-        <v>25</v>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Løbetur Z2 — 50 min, ratio 10/2</t>
+        </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>12/2</t>
+          <t>Marathon pace progression (25 min)</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Tempo-int.</t>
+          <t>22 km</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Peak long run – inkl. gangpauser. Fejr den!</t>
+          <t>Ratio 12/2 på lang tur.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="n">
+      <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>18/08 – 20/08 – 22/08</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>Taper</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>12/2</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>Let Z2</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>Taper start</t>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Løbetur Z2 — 50 min, ratio 10/2</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Marathon pace (30 min)</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>25 km</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>PEAK lang tur — ratio 12/2.</t>
         </is>
       </c>
     </row>
@@ -897,22 +923,24 @@
           <t>Taper</t>
         </is>
       </c>
-      <c r="D13" s="4" t="n">
-        <v>12</v>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Let løbetur — 35 min, ratio 12/2</t>
+        </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>12/2</t>
+          <t>Marathon pace kort (15 min)</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Marathon pace</t>
+          <t>15 km</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Marathon pace-stykke tirsdag</t>
+          <t>Taper start.</t>
         </is>
       </c>
     </row>
@@ -930,22 +958,24 @@
           <t>Race</t>
         </is>
       </c>
-      <c r="D14" s="5" t="n">
-        <v>8</v>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Let løbetur — 25 min, ratio 8/2</t>
+        </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>12/2</t>
+          <t>Aktivering — 20 min</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Let Z2</t>
+          <t>RACE</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>RACE DAY: Marathon du Médoc, 5. sept – 6:00-6:30/km, fase 2 fra 25 km: nyd det</t>
+          <t>RACE DAY 5/9: 6:00-6:30/km, gangpause hvert 12. min til km 25, derefter fri.</t>
         </is>
       </c>
     </row>
@@ -960,7 +990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1047,7 +1077,11 @@
           <t>5:35 – 6:24/km</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr"/>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Fra uge 3 (tempo intervals)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -1086,32 +1120,49 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Max langt løb</t>
+          <t>Run/walk ratio</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>25 km inkl. gangpauser</t>
+          <t>6/2 → 8/2 → 10/2 → 12/2</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Svarer til ~20-22 km løbebelastning</t>
+          <t>Se Oversigt-ark for uge-for-uge progression</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
+          <t>Peak lang tur</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>25 km (uge 11), inkl. gangpauser</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Svarer til ~20-22 km løbebelastning</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
           <t>Race</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Marathon du Médoc, 5. sept 2026</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Bordeaux</t>
         </is>

</xml_diff>